<commit_message>
minor updates, includes more complete units and implimentation of plotting IC/ICPMS data
</commit_message>
<xml_diff>
--- a/data/sampling/units.xlsx
+++ b/data/sampling/units.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/ECM/alhic1901_deep_layering/github/data/sampling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EBC434-ED91-7540-A75B-6CA9472C57B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB7759-28E7-5041-BE31-F7EC5B052D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1020" yWindow="760" windowWidth="29220" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="86">
   <si>
     <t>simple_name</t>
   </si>
@@ -122,10 +123,178 @@
     <t>Ca+</t>
   </si>
   <si>
-    <t>Ca$^+$</t>
-  </si>
-  <si>
-    <t>μg/L</t>
+    <t>Ca$^2+$</t>
+  </si>
+  <si>
+    <t>NO3-</t>
+  </si>
+  <si>
+    <t>SO42-</t>
+  </si>
+  <si>
+    <t>Na+</t>
+  </si>
+  <si>
+    <t>K+</t>
+  </si>
+  <si>
+    <t>Mg2+</t>
+  </si>
+  <si>
+    <t>SO$_4^{2-}$</t>
+  </si>
+  <si>
+    <t>NO$_3^-$</t>
+  </si>
+  <si>
+    <t>Na$^+$</t>
+  </si>
+  <si>
+    <t>K$^+$</t>
+  </si>
+  <si>
+    <t>Mg$^{2+}</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>* need to check units / Jacob</t>
+  </si>
+  <si>
+    <t>Li</t>
+  </si>
+  <si>
+    <t>Rb</t>
+  </si>
+  <si>
+    <t>Sr</t>
+  </si>
+  <si>
+    <t>Cd</t>
+  </si>
+  <si>
+    <t>Cs</t>
+  </si>
+  <si>
+    <t>Ba</t>
+  </si>
+  <si>
+    <t>La</t>
+  </si>
+  <si>
+    <t>Pr</t>
+  </si>
+  <si>
+    <t>Nd</t>
+  </si>
+  <si>
+    <t>Sm</t>
+  </si>
+  <si>
+    <t>Eu</t>
+  </si>
+  <si>
+    <t>Tb</t>
+  </si>
+  <si>
+    <t>Gd</t>
+  </si>
+  <si>
+    <t>Dy</t>
+  </si>
+  <si>
+    <t>Ho</t>
+  </si>
+  <si>
+    <t>Er</t>
+  </si>
+  <si>
+    <t>Tm</t>
+  </si>
+  <si>
+    <t>Yb</t>
+  </si>
+  <si>
+    <t>Lu</t>
+  </si>
+  <si>
+    <t>Pb</t>
+  </si>
+  <si>
+    <t>Th</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>Cr</t>
+  </si>
+  <si>
+    <t>As</t>
+  </si>
+  <si>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>Co</t>
+  </si>
+  <si>
+    <t>Ni</t>
+  </si>
+  <si>
+    <t>Cu</t>
+  </si>
+  <si>
+    <t>Zn</t>
+  </si>
+  <si>
+    <t>Mg</t>
+  </si>
+  <si>
+    <t>Al</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Ti</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Be</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>Zr</t>
+  </si>
+  <si>
+    <t>Mo</t>
+  </si>
+  <si>
+    <t>Ce</t>
+  </si>
+  <si>
+    <t>ng/L</t>
+  </si>
+  <si>
+    <t>µg/L</t>
+  </si>
+  <si>
+    <t>ug/L</t>
   </si>
 </sst>
 </file>
@@ -497,10 +666,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA282E54-A88C-8E4B-A9AB-DECBBDBF30F2}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -510,8 +679,11 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -522,7 +694,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -533,7 +705,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -544,7 +716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -555,7 +727,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -566,7 +738,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -577,7 +749,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -588,7 +760,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -599,52 +771,596 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" t="s">
+        <v>62</v>
+      </c>
+      <c r="C34" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" t="s">
+        <v>63</v>
+      </c>
+      <c r="C43" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>64</v>
+      </c>
+      <c r="B44" t="s">
+        <v>64</v>
+      </c>
+      <c r="C44" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>24</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B46" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B49" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>70</v>
+      </c>
+      <c r="B50" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>75</v>
+      </c>
+      <c r="B51" t="s">
+        <v>75</v>
+      </c>
+      <c r="C51" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>79</v>
+      </c>
+      <c r="B52" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>76</v>
+      </c>
+      <c r="B53" t="s">
+        <v>76</v>
+      </c>
+      <c r="C53" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>65</v>
+      </c>
+      <c r="B54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C54" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>27</v>
+      </c>
+      <c r="B55" t="s">
+        <v>28</v>
+      </c>
+      <c r="C55" t="s">
+        <v>7</v>
+      </c>
+      <c r="D55" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B56" t="s">
+        <v>35</v>
+      </c>
+      <c r="C56" t="s">
         <v>7</v>
+      </c>
+      <c r="D56" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>30</v>
+      </c>
+      <c r="B57" t="s">
+        <v>34</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>31</v>
+      </c>
+      <c r="B58" t="s">
+        <v>36</v>
+      </c>
+      <c r="C58" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>32</v>
+      </c>
+      <c r="B59" t="s">
+        <v>37</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>33</v>
+      </c>
+      <c r="B60" t="s">
+        <v>38</v>
+      </c>
+      <c r="C60" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DBBFFF1-1513-1440-994D-A2F6AD86A598}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update CFA data, integrate into plotting script
</commit_message>
<xml_diff>
--- a/data/sampling/units.xlsx
+++ b/data/sampling/units.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA110EC-53D6-264A-B547-9F048F54E70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07588A98-43D4-E543-B66E-9225B497835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="460" yWindow="760" windowWidth="29220" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
+    <workbookView xWindow="1000" yWindow="760" windowWidth="29220" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
update cc data with new fix from Jacob. Start making paper-ready figures
</commit_message>
<xml_diff>
--- a/data/sampling/units.xlsx
+++ b/data/sampling/units.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07588A98-43D4-E543-B66E-9225B497835C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1B4CD3-32FD-CE4D-BD3A-4180F7F3AE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1000" yWindow="760" windowWidth="29220" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
+    <workbookView xWindow="1080" yWindow="760" windowWidth="29160" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -93,9 +93,6 @@
     <t>Ar Age</t>
   </si>
   <si>
-    <t>kyr</t>
-  </si>
-  <si>
     <t>concentration</t>
   </si>
   <si>
@@ -307,6 +304,9 @@
   </si>
   <si>
     <t>$\delta^{13}C$</t>
+  </si>
+  <si>
+    <t>Ma</t>
   </si>
 </sst>
 </file>
@@ -692,7 +692,7 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -741,10 +741,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" t="s">
         <v>88</v>
-      </c>
-      <c r="B6" t="s">
-        <v>89</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -769,15 +769,15 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
@@ -785,600 +785,600 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C41" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C44" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B46" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B49" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C50" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B52" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C52" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C53" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C54" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C55" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B56" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B57" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C57" t="s">
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B58" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C58" t="s">
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B59" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C59" t="s">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B60" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C60" t="s">
         <v>7</v>
       </c>
       <c r="D60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C61" t="s">
         <v>7</v>
       </c>
       <c r="D61" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
+        <v>84</v>
+      </c>
+      <c r="B62" t="s">
         <v>85</v>
-      </c>
-      <c r="B62" t="s">
-        <v>86</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
add new IC data from section 230_4
</commit_message>
<xml_diff>
--- a/data/sampling/units.xlsx
+++ b/data/sampling/units.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1B4CD3-32FD-CE4D-BD3A-4180F7F3AE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A005E79C-1FA2-2147-876C-4AE3FDC3C567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="760" windowWidth="29160" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
+    <workbookView xWindow="-280" yWindow="-20420" windowWidth="29160" windowHeight="18880" xr2:uid="{1EDB8023-74AD-8E40-8F17-4D0EA63C8EF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="91">
   <si>
     <t>simple_name</t>
   </si>
@@ -150,9 +150,6 @@
     <t>notes</t>
   </si>
   <si>
-    <t>* need to check units / Jacob</t>
-  </si>
-  <si>
     <t>Li</t>
   </si>
   <si>
@@ -282,12 +279,6 @@
     <t>ng/L</t>
   </si>
   <si>
-    <t>µg/L</t>
-  </si>
-  <si>
-    <t>ug/L</t>
-  </si>
-  <si>
     <t>Ca$^{2+}$</t>
   </si>
   <si>
@@ -307,6 +298,18 @@
   </si>
   <si>
     <t>Ma</t>
+  </si>
+  <si>
+    <t>$\mu g L^{-1}$</t>
+  </si>
+  <si>
+    <t>ng $L^{-1}$</t>
+  </si>
+  <si>
+    <t>NH4+</t>
+  </si>
+  <si>
+    <t>NH$_4^+$</t>
   </si>
 </sst>
 </file>
@@ -678,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA282E54-A88C-8E4B-A9AB-DECBBDBF30F2}">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -741,10 +744,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -769,7 +772,7 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -780,7 +783,7 @@
         <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -796,299 +799,299 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C20" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C26" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C34" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C35" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C37" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
@@ -1099,40 +1102,40 @@
         <v>25</v>
       </c>
       <c r="C38" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B39" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C39" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C41" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
@@ -1143,51 +1146,51 @@
         <v>24</v>
       </c>
       <c r="C42" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C43" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C44" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
@@ -1198,112 +1201,109 @@
         <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>64</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>64</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>71</v>
+      </c>
+      <c r="B52" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>75</v>
+      </c>
+      <c r="B53" t="s">
+        <v>75</v>
+      </c>
+      <c r="C53" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>72</v>
+      </c>
+      <c r="B54" t="s">
+        <v>72</v>
+      </c>
+      <c r="C54" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>61</v>
+      </c>
+      <c r="B55" t="s">
+        <v>61</v>
+      </c>
+      <c r="C55" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>83</v>
+      </c>
+      <c r="B56" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>65</v>
-      </c>
-      <c r="B49" t="s">
-        <v>65</v>
-      </c>
-      <c r="C49" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>66</v>
-      </c>
-      <c r="B50" t="s">
-        <v>66</v>
-      </c>
-      <c r="C50" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>67</v>
-      </c>
-      <c r="B51" t="s">
-        <v>67</v>
-      </c>
-      <c r="C51" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>72</v>
-      </c>
-      <c r="B52" t="s">
-        <v>72</v>
-      </c>
-      <c r="C52" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>76</v>
-      </c>
-      <c r="B53" t="s">
-        <v>76</v>
-      </c>
-      <c r="C53" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>73</v>
-      </c>
-      <c r="B54" t="s">
-        <v>73</v>
-      </c>
-      <c r="C54" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" t="s">
-        <v>62</v>
-      </c>
-      <c r="C55" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>86</v>
-      </c>
-      <c r="B56" t="s">
-        <v>83</v>
-      </c>
       <c r="C56" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>26</v>
       </c>
@@ -1311,13 +1311,10 @@
         <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>27</v>
       </c>
@@ -1325,13 +1322,10 @@
         <v>31</v>
       </c>
       <c r="C58" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>28</v>
       </c>
@@ -1339,13 +1333,10 @@
         <v>33</v>
       </c>
       <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>29</v>
       </c>
@@ -1353,13 +1344,10 @@
         <v>34</v>
       </c>
       <c r="C60" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>30</v>
       </c>
@@ -1367,21 +1355,29 @@
         <v>35</v>
       </c>
       <c r="C61" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B62" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C62" t="s">
-        <v>7</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B63" t="s">
+        <v>90</v>
+      </c>
+      <c r="C63" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>